<commit_message>
feat: rebrand the product as Veyrafy with the new logo
- Every customer-visible text says Veyrafy: the homepage, the app, questions
  and decisions, messages and errors, toasts, Veyrafy Operations, exports and
  import templates (regenerated: Veyrafy-Master-Data-Import.xlsx), page title.
- New mark: three strokes fanning into a green check, redrawn as a vector from
  the supplied artwork (docs/brand-logo.png), with an inverse variant for dark
  backgrounds; new favicon.
- Unchanged on purpose: the internal code name veyra (packages, VEYRA_*
  environment variables, session cookie, VEYRA_ADMIN role, databases), so no
  deployment reconfiguration or forced sign-out; and the fictional demo buyer
  "Veyra Demo Industries Pvt Ltd", printed inside the sample invoices.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MJDS4UpCHTEKiWMJzVRoAM
</commit_message>
<xml_diff>
--- a/fixtures/imports/templates/GoodsReceiptLines.xlsx
+++ b/fixtures/imports/templates/GoodsReceiptLines.xlsx
@@ -67,14 +67,14 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Veyra business records: Goods receipt lines</t>
+          <t xml:space="preserve">Veyrafy business records: Goods receipt lines</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">Fill in one row per record on the sheet(s) of this workbook, then upload the file in Veyra under ERP → Import and export.</t>
+          <t xml:space="preserve">Fill in one row per record on the sheet(s) of this workbook, then upload the file in Veyrafy under ERP → Import and export.</t>
         </is>
       </c>
     </row>
@@ -88,14 +88,14 @@
     <row r="4">
       <c r="A4" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">Veyra checks the whole upload before anything is imported. If any row has a problem, nothing is imported: fix the rows it lists and upload again.</t>
+          <t xml:space="preserve">Veyrafy checks the whole upload before anything is imported. If any row has a problem, nothing is imported: fix the rows it lists and upload again.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr" s="3">
         <is>
-          <t xml:space="preserve">Records that already exist with the same details are skipped. Veyra never changes an existing record.</t>
+          <t xml:space="preserve">Records that already exist with the same details are skipped. Veyrafy never changes an existing record.</t>
         </is>
       </c>
     </row>

</xml_diff>